<commit_message>
Feature good practices interop #2
suppression type.coding.system 095cb4aedf9fda767a1d7d838a1e01301240d53e
</commit_message>
<xml_diff>
--- a/ig/feature-good-practices-interop/StructureDefinition-as-device.xlsx
+++ b/ig/feature-good-practices-interop/StructureDefinition-as-device.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3153" uniqueCount="492">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2764" uniqueCount="440">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-04-05T15:55:13+00:00</t>
+    <t>2023-04-05T16:00:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1111,163 +1111,6 @@
   </si>
   <si>
     <t>https://mos.esante.gouv.fr/NOS/JDV_J135-EquipementMaterielLourd-RASS/FHIR/JDV-J135-EquipementMaterielLourd-RASS</t>
-  </si>
-  <si>
-    <t>Device.type.id</t>
-  </si>
-  <si>
-    <t>Device.type.extension</t>
-  </si>
-  <si>
-    <t>Device.type.coding</t>
-  </si>
-  <si>
-    <t>Code defined by a terminology system</t>
-  </si>
-  <si>
-    <t>A reference to a code defined by a terminology system.</t>
-  </si>
-  <si>
-    <t>Codes may be defined very casually in enumerations, or code lists, up to very formal definitions such as SNOMED CT - see the HL7 v3 Core Principles for more information.  Ordering of codings is undefined and SHALL NOT be used to infer meaning. Generally, at most only one of the coding values will be labeled as UserSelected = true.</t>
-  </si>
-  <si>
-    <t>Allows for alternative encodings within a code system, and translations to other code systems.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding</t>
-  </si>
-  <si>
-    <t>union(., ./translation)</t>
-  </si>
-  <si>
-    <t>Device.type.coding.id</t>
-  </si>
-  <si>
-    <t>Device.type.coding.extension</t>
-  </si>
-  <si>
-    <t>Device.type.coding.system</t>
-  </si>
-  <si>
-    <t>Identity of the terminology system</t>
-  </si>
-  <si>
-    <t>The identification of the code system that defines the meaning of the symbol in the code.</t>
-  </si>
-  <si>
-    <t>The URI may be an OID (urn:oid:...) or a UUID (urn:uuid:...).  OIDs and UUIDs SHALL be references to the HL7 OID registry. Otherwise, the URI should come from HL7's list of FHIR defined special URIs or it should reference to some definition that establishes the system clearly and unambiguously.</t>
-  </si>
-  <si>
-    <t>Need to be unambiguous about the source of the definition of the symbol.</t>
-  </si>
-  <si>
-    <t>https://mos.esante.gouv.fr/NOS/TRE_R272-EquipementMaterielLourd/FHIR/TRE-R272-EquipementMaterielLourd</t>
-  </si>
-  <si>
-    <t>Coding.system</t>
-  </si>
-  <si>
-    <t>./codeSystem</t>
-  </si>
-  <si>
-    <t>Device.type.coding.version</t>
-  </si>
-  <si>
-    <t>Version of the system - if relevant</t>
-  </si>
-  <si>
-    <t>The version of the code system which was used when choosing this code. Note that a well-maintained code system does not need the version reported, because the meaning of codes is consistent across versions. However this cannot consistently be assured, and when the meaning is not guaranteed to be consistent, the version SHOULD be exchanged.</t>
-  </si>
-  <si>
-    <t>Where the terminology does not clearly define what string should be used to identify code system versions, the recommendation is to use the date (expressed in FHIR date format) on which that version was officially published as the version date.</t>
-  </si>
-  <si>
-    <t>Coding.version</t>
-  </si>
-  <si>
-    <t>./codeSystemVersion</t>
-  </si>
-  <si>
-    <t>Device.type.coding.code</t>
-  </si>
-  <si>
-    <t>Symbol in syntax defined by the system</t>
-  </si>
-  <si>
-    <t>A symbol in syntax defined by the system. The symbol may be a predefined code or an expression in a syntax defined by the coding system (e.g. post-coordination).</t>
-  </si>
-  <si>
-    <t>Need to refer to a particular code in the system.</t>
-  </si>
-  <si>
-    <t>Coding.code</t>
-  </si>
-  <si>
-    <t>./code</t>
-  </si>
-  <si>
-    <t>Device.type.coding.display</t>
-  </si>
-  <si>
-    <t>Representation defined by the system</t>
-  </si>
-  <si>
-    <t>A representation of the meaning of the code in the system, following the rules of the system.</t>
-  </si>
-  <si>
-    <t>Need to be able to carry a human-readable meaning of the code for readers that do not know  the system.</t>
-  </si>
-  <si>
-    <t>Coding.display</t>
-  </si>
-  <si>
-    <t>CV.displayName</t>
-  </si>
-  <si>
-    <t>Device.type.coding.userSelected</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boolean
-</t>
-  </si>
-  <si>
-    <t>If this coding was chosen directly by the user</t>
-  </si>
-  <si>
-    <t>Indicates that this coding was chosen by a user directly - e.g. off a pick list of available items (codes or displays).</t>
-  </si>
-  <si>
-    <t>Amongst a set of alternatives, a directly chosen code is the most appropriate starting point for new translations. There is some ambiguity about what exactly 'directly chosen' implies, and trading partner agreement may be needed to clarify the use of this element and its consequences more completely.</t>
-  </si>
-  <si>
-    <t>This has been identified as a clinical safety criterium - that this exact system/code pair was chosen explicitly, rather than inferred by the system based on some rules or language processing.</t>
-  </si>
-  <si>
-    <t>Coding.userSelected</t>
-  </si>
-  <si>
-    <t>CD.codingRationale</t>
-  </si>
-  <si>
-    <t>Device.type.text</t>
-  </si>
-  <si>
-    <t>Plain text representation of the concept</t>
-  </si>
-  <si>
-    <t>A human language representation of the concept as seen/selected/uttered by the user who entered the data and/or which represents the intended meaning of the user.</t>
-  </si>
-  <si>
-    <t>Very often the text is the same as a displayName of one of the codings.</t>
-  </si>
-  <si>
-    <t>The codes from the terminologies do not always capture the correct meaning with all the nuances of the human using them, or sometimes there is no appropriate code at all. In these cases, the text is used to capture the full meaning of the source.</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>./originalText[mediaType/code="text/plain"]/data</t>
   </si>
   <si>
     <t>Device.specialization</t>
@@ -1849,7 +1692,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AM89"/>
+  <dimension ref="A1:AM78"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="44.8515625" customWidth="true" bestFit="true"/>
@@ -7460,7 +7303,7 @@
         <v>75</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>74</v>
@@ -7472,13 +7315,13 @@
         <v>74</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>97</v>
+        <v>220</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>98</v>
+        <v>348</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>99</v>
+        <v>349</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -7529,19 +7372,19 @@
         <v>74</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>100</v>
+        <v>347</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI51" t="s" s="2">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="AJ51" t="s" s="2">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="AK51" t="s" s="2">
         <v>101</v>
@@ -7555,21 +7398,21 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="E52" s="2"/>
       <c r="F52" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G52" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H52" t="s" s="2">
         <v>74</v>
@@ -7581,17 +7424,15 @@
         <v>74</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>105</v>
+        <v>98</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="N52" t="s" s="2">
-        <v>107</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="N52" s="2"/>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
         <v>74</v>
@@ -7628,34 +7469,34 @@
         <v>74</v>
       </c>
       <c r="AB52" t="s" s="2">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="AC52" t="s" s="2">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="AD52" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE52" t="s" s="2">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH52" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI52" t="s" s="2">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="AJ52" t="s" s="2">
-        <v>112</v>
+        <v>74</v>
       </c>
       <c r="AK52" t="s" s="2">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="AL52" t="s" s="2">
         <v>74</v>
@@ -7666,14 +7507,14 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E53" s="2"/>
       <c r="F53" t="s" s="2">
@@ -7689,23 +7530,21 @@
         <v>74</v>
       </c>
       <c r="J53" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>137</v>
+        <v>104</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>350</v>
+        <v>105</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>351</v>
+        <v>106</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>352</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>353</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
         <v>74</v>
       </c>
@@ -7741,19 +7580,19 @@
         <v>74</v>
       </c>
       <c r="AB53" t="s" s="2">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="AC53" t="s" s="2">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="AD53" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE53" t="s" s="2">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>354</v>
+        <v>111</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>75</v>
@@ -7765,10 +7604,10 @@
         <v>93</v>
       </c>
       <c r="AJ53" t="s" s="2">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="AK53" t="s" s="2">
-        <v>355</v>
+        <v>95</v>
       </c>
       <c r="AL53" t="s" s="2">
         <v>74</v>
@@ -7779,42 +7618,46 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>356</v>
+        <v>352</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
-        <v>74</v>
+        <v>228</v>
       </c>
       <c r="E54" s="2"/>
       <c r="F54" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>74</v>
       </c>
       <c r="I54" t="s" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>98</v>
+        <v>229</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
+        <v>230</v>
+      </c>
+      <c r="N54" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="O54" t="s" s="2">
+        <v>202</v>
+      </c>
       <c r="P54" t="s" s="2">
         <v>74</v>
       </c>
@@ -7862,22 +7705,22 @@
         <v>74</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>100</v>
+        <v>231</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI54" t="s" s="2">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="AJ54" t="s" s="2">
-        <v>74</v>
+        <v>112</v>
       </c>
       <c r="AK54" t="s" s="2">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="AL54" t="s" s="2">
         <v>74</v>
@@ -7888,21 +7731,21 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>357</v>
+        <v>353</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
-        <v>103</v>
+        <v>326</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>74</v>
@@ -7914,16 +7757,16 @@
         <v>74</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>104</v>
+        <v>282</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>105</v>
+        <v>354</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>106</v>
+        <v>355</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>107</v>
+        <v>285</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -7961,34 +7804,34 @@
         <v>74</v>
       </c>
       <c r="AB55" t="s" s="2">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="AC55" t="s" s="2">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="AD55" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE55" t="s" s="2">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>111</v>
+        <v>353</v>
       </c>
       <c r="AG55" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AH55" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI55" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="AK55" t="s" s="2">
-        <v>95</v>
+        <v>288</v>
       </c>
       <c r="AL55" t="s" s="2">
         <v>74</v>
@@ -7999,10 +7842,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8022,29 +7865,27 @@
         <v>74</v>
       </c>
       <c r="J56" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K56" t="s" s="2">
-        <v>125</v>
+        <v>97</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>361</v>
-      </c>
-      <c r="O56" t="s" s="2">
-        <v>362</v>
-      </c>
+        <v>236</v>
+      </c>
+      <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>74</v>
       </c>
       <c r="Q56" s="2"/>
       <c r="R56" t="s" s="2">
-        <v>363</v>
+        <v>74</v>
       </c>
       <c r="S56" t="s" s="2">
         <v>74</v>
@@ -8086,7 +7927,7 @@
         <v>74</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>364</v>
+        <v>356</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>75</v>
@@ -8101,10 +7942,10 @@
         <v>94</v>
       </c>
       <c r="AK56" t="s" s="2">
-        <v>365</v>
+        <v>101</v>
       </c>
       <c r="AL56" t="s" s="2">
-        <v>74</v>
+        <v>238</v>
       </c>
       <c r="AM56" t="s" s="2">
         <v>74</v>
@@ -8112,10 +7953,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>366</v>
+        <v>359</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8126,7 +7967,7 @@
         <v>75</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>74</v>
@@ -8135,20 +7976,18 @@
         <v>74</v>
       </c>
       <c r="J57" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>97</v>
+        <v>220</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>367</v>
+        <v>360</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>368</v>
-      </c>
-      <c r="N57" t="s" s="2">
-        <v>369</v>
-      </c>
+        <v>361</v>
+      </c>
+      <c r="N57" s="2"/>
       <c r="O57" s="2"/>
       <c r="P57" t="s" s="2">
         <v>74</v>
@@ -8197,13 +8036,13 @@
         <v>74</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>370</v>
+        <v>359</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH57" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI57" t="s" s="2">
         <v>93</v>
@@ -8212,7 +8051,7 @@
         <v>94</v>
       </c>
       <c r="AK57" t="s" s="2">
-        <v>371</v>
+        <v>101</v>
       </c>
       <c r="AL57" t="s" s="2">
         <v>74</v>
@@ -8223,10 +8062,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8246,23 +8085,19 @@
         <v>74</v>
       </c>
       <c r="J58" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>160</v>
+        <v>97</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>373</v>
+        <v>98</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>374</v>
-      </c>
-      <c r="N58" t="s" s="2">
-        <v>236</v>
-      </c>
-      <c r="O58" t="s" s="2">
-        <v>375</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="N58" s="2"/>
+      <c r="O58" s="2"/>
       <c r="P58" t="s" s="2">
         <v>74</v>
       </c>
@@ -8310,7 +8145,7 @@
         <v>74</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>376</v>
+        <v>100</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>75</v>
@@ -8319,13 +8154,13 @@
         <v>81</v>
       </c>
       <c r="AI58" t="s" s="2">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="AJ58" t="s" s="2">
-        <v>94</v>
+        <v>74</v>
       </c>
       <c r="AK58" t="s" s="2">
-        <v>377</v>
+        <v>101</v>
       </c>
       <c r="AL58" t="s" s="2">
         <v>74</v>
@@ -8336,21 +8171,21 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>378</v>
+        <v>363</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
-        <v>74</v>
+        <v>103</v>
       </c>
       <c r="E59" s="2"/>
       <c r="F59" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G59" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H59" t="s" s="2">
         <v>74</v>
@@ -8359,23 +8194,21 @@
         <v>74</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>379</v>
+        <v>105</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>380</v>
+        <v>106</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>236</v>
-      </c>
-      <c r="O59" t="s" s="2">
-        <v>381</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="O59" s="2"/>
       <c r="P59" t="s" s="2">
         <v>74</v>
       </c>
@@ -8411,34 +8244,34 @@
         <v>74</v>
       </c>
       <c r="AB59" t="s" s="2">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="AC59" t="s" s="2">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="AD59" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE59" t="s" s="2">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>382</v>
+        <v>111</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH59" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI59" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ59" t="s" s="2">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="AK59" t="s" s="2">
-        <v>383</v>
+        <v>95</v>
       </c>
       <c r="AL59" t="s" s="2">
         <v>74</v>
@@ -8449,45 +8282,45 @@
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>384</v>
+        <v>364</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>384</v>
+        <v>364</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>74</v>
+        <v>228</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>74</v>
       </c>
       <c r="I60" t="s" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="J60" t="s" s="2">
         <v>82</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>385</v>
+        <v>104</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>386</v>
+        <v>229</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>387</v>
+        <v>230</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>388</v>
+        <v>107</v>
       </c>
       <c r="O60" t="s" s="2">
-        <v>389</v>
+        <v>202</v>
       </c>
       <c r="P60" t="s" s="2">
         <v>74</v>
@@ -8536,22 +8369,22 @@
         <v>74</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>390</v>
+        <v>231</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI60" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ60" t="s" s="2">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="AK60" t="s" s="2">
-        <v>391</v>
+        <v>95</v>
       </c>
       <c r="AL60" t="s" s="2">
         <v>74</v>
@@ -8562,14 +8395,14 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>392</v>
+        <v>365</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>392</v>
+        <v>365</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>74</v>
+        <v>326</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -8585,23 +8418,21 @@
         <v>74</v>
       </c>
       <c r="J61" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>97</v>
+        <v>282</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>393</v>
+        <v>366</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>394</v>
+        <v>367</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>395</v>
-      </c>
-      <c r="O61" t="s" s="2">
-        <v>396</v>
-      </c>
+        <v>285</v>
+      </c>
+      <c r="O61" s="2"/>
       <c r="P61" t="s" s="2">
         <v>74</v>
       </c>
@@ -8649,7 +8480,7 @@
         <v>74</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>397</v>
+        <v>365</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>75</v>
@@ -8664,7 +8495,7 @@
         <v>94</v>
       </c>
       <c r="AK61" t="s" s="2">
-        <v>398</v>
+        <v>288</v>
       </c>
       <c r="AL61" t="s" s="2">
         <v>74</v>
@@ -8675,10 +8506,10 @@
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>399</v>
+        <v>368</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>399</v>
+        <v>368</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -8689,7 +8520,7 @@
         <v>75</v>
       </c>
       <c r="G62" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H62" t="s" s="2">
         <v>74</v>
@@ -8701,13 +8532,13 @@
         <v>74</v>
       </c>
       <c r="K62" t="s" s="2">
-        <v>220</v>
+        <v>205</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>400</v>
+        <v>369</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>401</v>
+        <v>370</v>
       </c>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
@@ -8758,13 +8589,13 @@
         <v>74</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>399</v>
+        <v>368</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH62" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI62" t="s" s="2">
         <v>93</v>
@@ -8773,10 +8604,10 @@
         <v>94</v>
       </c>
       <c r="AK62" t="s" s="2">
-        <v>101</v>
+        <v>371</v>
       </c>
       <c r="AL62" t="s" s="2">
-        <v>74</v>
+        <v>238</v>
       </c>
       <c r="AM62" t="s" s="2">
         <v>74</v>
@@ -8784,10 +8615,10 @@
     </row>
     <row r="63">
       <c r="A63" t="s" s="2">
-        <v>402</v>
+        <v>372</v>
       </c>
       <c r="B63" t="s" s="2">
-        <v>402</v>
+        <v>372</v>
       </c>
       <c r="C63" s="2"/>
       <c r="D63" t="s" s="2">
@@ -8795,7 +8626,7 @@
       </c>
       <c r="E63" s="2"/>
       <c r="F63" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G63" t="s" s="2">
         <v>81</v>
@@ -8813,12 +8644,14 @@
         <v>97</v>
       </c>
       <c r="L63" t="s" s="2">
-        <v>98</v>
+        <v>373</v>
       </c>
       <c r="M63" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N63" s="2"/>
+        <v>374</v>
+      </c>
+      <c r="N63" t="s" s="2">
+        <v>236</v>
+      </c>
       <c r="O63" s="2"/>
       <c r="P63" t="s" s="2">
         <v>74</v>
@@ -8867,19 +8700,19 @@
         <v>74</v>
       </c>
       <c r="AF63" t="s" s="2">
-        <v>100</v>
+        <v>372</v>
       </c>
       <c r="AG63" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AH63" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AI63" t="s" s="2">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="AJ63" t="s" s="2">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="AK63" t="s" s="2">
         <v>101</v>
@@ -8893,21 +8726,21 @@
     </row>
     <row r="64">
       <c r="A64" t="s" s="2">
-        <v>403</v>
+        <v>375</v>
       </c>
       <c r="B64" t="s" s="2">
-        <v>403</v>
+        <v>375</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" t="s" s="2">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="E64" s="2"/>
       <c r="F64" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G64" t="s" s="2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H64" t="s" s="2">
         <v>74</v>
@@ -8919,17 +8752,15 @@
         <v>74</v>
       </c>
       <c r="K64" t="s" s="2">
-        <v>104</v>
+        <v>220</v>
       </c>
       <c r="L64" t="s" s="2">
-        <v>105</v>
+        <v>376</v>
       </c>
       <c r="M64" t="s" s="2">
-        <v>106</v>
-      </c>
-      <c r="N64" t="s" s="2">
-        <v>107</v>
-      </c>
+        <v>377</v>
+      </c>
+      <c r="N64" s="2"/>
       <c r="O64" s="2"/>
       <c r="P64" t="s" s="2">
         <v>74</v>
@@ -8966,19 +8797,19 @@
         <v>74</v>
       </c>
       <c r="AB64" t="s" s="2">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="AC64" t="s" s="2">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="AD64" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE64" t="s" s="2">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="AF64" t="s" s="2">
-        <v>111</v>
+        <v>375</v>
       </c>
       <c r="AG64" t="s" s="2">
         <v>75</v>
@@ -8990,10 +8821,10 @@
         <v>93</v>
       </c>
       <c r="AJ64" t="s" s="2">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="AK64" t="s" s="2">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="AL64" t="s" s="2">
         <v>74</v>
@@ -9004,46 +8835,42 @@
     </row>
     <row r="65">
       <c r="A65" t="s" s="2">
-        <v>404</v>
+        <v>378</v>
       </c>
       <c r="B65" t="s" s="2">
-        <v>404</v>
+        <v>378</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" t="s" s="2">
-        <v>228</v>
+        <v>74</v>
       </c>
       <c r="E65" s="2"/>
       <c r="F65" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G65" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H65" t="s" s="2">
         <v>74</v>
       </c>
       <c r="I65" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J65" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K65" t="s" s="2">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="L65" t="s" s="2">
-        <v>229</v>
+        <v>98</v>
       </c>
       <c r="M65" t="s" s="2">
-        <v>230</v>
-      </c>
-      <c r="N65" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="O65" t="s" s="2">
-        <v>202</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="N65" s="2"/>
+      <c r="O65" s="2"/>
       <c r="P65" t="s" s="2">
         <v>74</v>
       </c>
@@ -9091,22 +8918,22 @@
         <v>74</v>
       </c>
       <c r="AF65" t="s" s="2">
-        <v>231</v>
+        <v>100</v>
       </c>
       <c r="AG65" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH65" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI65" t="s" s="2">
-        <v>93</v>
+        <v>74</v>
       </c>
       <c r="AJ65" t="s" s="2">
-        <v>112</v>
+        <v>74</v>
       </c>
       <c r="AK65" t="s" s="2">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="AL65" t="s" s="2">
         <v>74</v>
@@ -9117,21 +8944,21 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="2">
-        <v>405</v>
+        <v>379</v>
       </c>
       <c r="B66" t="s" s="2">
-        <v>405</v>
+        <v>379</v>
       </c>
       <c r="C66" s="2"/>
       <c r="D66" t="s" s="2">
-        <v>326</v>
+        <v>103</v>
       </c>
       <c r="E66" s="2"/>
       <c r="F66" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="G66" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H66" t="s" s="2">
         <v>74</v>
@@ -9143,16 +8970,16 @@
         <v>74</v>
       </c>
       <c r="K66" t="s" s="2">
-        <v>282</v>
+        <v>104</v>
       </c>
       <c r="L66" t="s" s="2">
-        <v>406</v>
+        <v>105</v>
       </c>
       <c r="M66" t="s" s="2">
-        <v>407</v>
+        <v>106</v>
       </c>
       <c r="N66" t="s" s="2">
-        <v>285</v>
+        <v>107</v>
       </c>
       <c r="O66" s="2"/>
       <c r="P66" t="s" s="2">
@@ -9190,34 +9017,34 @@
         <v>74</v>
       </c>
       <c r="AB66" t="s" s="2">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="AC66" t="s" s="2">
-        <v>74</v>
+        <v>109</v>
       </c>
       <c r="AD66" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE66" t="s" s="2">
-        <v>74</v>
+        <v>110</v>
       </c>
       <c r="AF66" t="s" s="2">
-        <v>405</v>
+        <v>111</v>
       </c>
       <c r="AG66" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AH66" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI66" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ66" t="s" s="2">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="AK66" t="s" s="2">
-        <v>288</v>
+        <v>95</v>
       </c>
       <c r="AL66" t="s" s="2">
         <v>74</v>
@@ -9228,44 +9055,46 @@
     </row>
     <row r="67">
       <c r="A67" t="s" s="2">
-        <v>408</v>
+        <v>380</v>
       </c>
       <c r="B67" t="s" s="2">
-        <v>408</v>
+        <v>380</v>
       </c>
       <c r="C67" s="2"/>
       <c r="D67" t="s" s="2">
-        <v>74</v>
+        <v>228</v>
       </c>
       <c r="E67" s="2"/>
       <c r="F67" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G67" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H67" t="s" s="2">
         <v>74</v>
       </c>
       <c r="I67" t="s" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="J67" t="s" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="K67" t="s" s="2">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="L67" t="s" s="2">
-        <v>409</v>
+        <v>229</v>
       </c>
       <c r="M67" t="s" s="2">
-        <v>410</v>
+        <v>230</v>
       </c>
       <c r="N67" t="s" s="2">
-        <v>236</v>
-      </c>
-      <c r="O67" s="2"/>
+        <v>107</v>
+      </c>
+      <c r="O67" t="s" s="2">
+        <v>202</v>
+      </c>
       <c r="P67" t="s" s="2">
         <v>74</v>
       </c>
@@ -9313,25 +9142,25 @@
         <v>74</v>
       </c>
       <c r="AF67" t="s" s="2">
-        <v>408</v>
+        <v>231</v>
       </c>
       <c r="AG67" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH67" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI67" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ67" t="s" s="2">
-        <v>94</v>
+        <v>112</v>
       </c>
       <c r="AK67" t="s" s="2">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="AL67" t="s" s="2">
-        <v>238</v>
+        <v>74</v>
       </c>
       <c r="AM67" t="s" s="2">
         <v>74</v>
@@ -9339,10 +9168,10 @@
     </row>
     <row r="68">
       <c r="A68" t="s" s="2">
-        <v>411</v>
+        <v>381</v>
       </c>
       <c r="B68" t="s" s="2">
-        <v>411</v>
+        <v>381</v>
       </c>
       <c r="C68" s="2"/>
       <c r="D68" t="s" s="2">
@@ -9350,10 +9179,10 @@
       </c>
       <c r="E68" s="2"/>
       <c r="F68" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="G68" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="H68" t="s" s="2">
         <v>74</v>
@@ -9365,15 +9194,17 @@
         <v>74</v>
       </c>
       <c r="K68" t="s" s="2">
-        <v>220</v>
+        <v>282</v>
       </c>
       <c r="L68" t="s" s="2">
-        <v>412</v>
+        <v>382</v>
       </c>
       <c r="M68" t="s" s="2">
-        <v>413</v>
-      </c>
-      <c r="N68" s="2"/>
+        <v>383</v>
+      </c>
+      <c r="N68" t="s" s="2">
+        <v>285</v>
+      </c>
       <c r="O68" s="2"/>
       <c r="P68" t="s" s="2">
         <v>74</v>
@@ -9422,13 +9253,13 @@
         <v>74</v>
       </c>
       <c r="AF68" t="s" s="2">
-        <v>411</v>
+        <v>381</v>
       </c>
       <c r="AG68" t="s" s="2">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="AH68" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI68" t="s" s="2">
         <v>93</v>
@@ -9437,7 +9268,7 @@
         <v>94</v>
       </c>
       <c r="AK68" t="s" s="2">
-        <v>101</v>
+        <v>288</v>
       </c>
       <c r="AL68" t="s" s="2">
         <v>74</v>
@@ -9448,10 +9279,10 @@
     </row>
     <row r="69">
       <c r="A69" t="s" s="2">
-        <v>414</v>
+        <v>384</v>
       </c>
       <c r="B69" t="s" s="2">
-        <v>414</v>
+        <v>384</v>
       </c>
       <c r="C69" s="2"/>
       <c r="D69" t="s" s="2">
@@ -9462,7 +9293,7 @@
         <v>75</v>
       </c>
       <c r="G69" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="H69" t="s" s="2">
         <v>74</v>
@@ -9474,15 +9305,17 @@
         <v>74</v>
       </c>
       <c r="K69" t="s" s="2">
-        <v>97</v>
+        <v>385</v>
       </c>
       <c r="L69" t="s" s="2">
-        <v>98</v>
+        <v>386</v>
       </c>
       <c r="M69" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N69" s="2"/>
+        <v>387</v>
+      </c>
+      <c r="N69" t="s" s="2">
+        <v>388</v>
+      </c>
       <c r="O69" s="2"/>
       <c r="P69" t="s" s="2">
         <v>74</v>
@@ -9531,22 +9364,22 @@
         <v>74</v>
       </c>
       <c r="AF69" t="s" s="2">
-        <v>100</v>
+        <v>384</v>
       </c>
       <c r="AG69" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH69" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI69" t="s" s="2">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="AJ69" t="s" s="2">
-        <v>74</v>
+        <v>389</v>
       </c>
       <c r="AK69" t="s" s="2">
-        <v>101</v>
+        <v>390</v>
       </c>
       <c r="AL69" t="s" s="2">
         <v>74</v>
@@ -9557,14 +9390,14 @@
     </row>
     <row r="70">
       <c r="A70" t="s" s="2">
-        <v>415</v>
+        <v>391</v>
       </c>
       <c r="B70" t="s" s="2">
-        <v>415</v>
+        <v>391</v>
       </c>
       <c r="C70" s="2"/>
       <c r="D70" t="s" s="2">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="E70" s="2"/>
       <c r="F70" t="s" s="2">
@@ -9583,16 +9416,16 @@
         <v>74</v>
       </c>
       <c r="K70" t="s" s="2">
-        <v>104</v>
+        <v>282</v>
       </c>
       <c r="L70" t="s" s="2">
-        <v>105</v>
+        <v>392</v>
       </c>
       <c r="M70" t="s" s="2">
-        <v>106</v>
+        <v>393</v>
       </c>
       <c r="N70" t="s" s="2">
-        <v>107</v>
+        <v>285</v>
       </c>
       <c r="O70" s="2"/>
       <c r="P70" t="s" s="2">
@@ -9630,19 +9463,19 @@
         <v>74</v>
       </c>
       <c r="AB70" t="s" s="2">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="AC70" t="s" s="2">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="AD70" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE70" t="s" s="2">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="AF70" t="s" s="2">
-        <v>111</v>
+        <v>391</v>
       </c>
       <c r="AG70" t="s" s="2">
         <v>75</v>
@@ -9654,10 +9487,10 @@
         <v>93</v>
       </c>
       <c r="AJ70" t="s" s="2">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="AK70" t="s" s="2">
-        <v>95</v>
+        <v>288</v>
       </c>
       <c r="AL70" t="s" s="2">
         <v>74</v>
@@ -9668,45 +9501,45 @@
     </row>
     <row r="71">
       <c r="A71" t="s" s="2">
-        <v>416</v>
+        <v>394</v>
       </c>
       <c r="B71" t="s" s="2">
-        <v>416</v>
+        <v>394</v>
       </c>
       <c r="C71" s="2"/>
       <c r="D71" t="s" s="2">
-        <v>228</v>
+        <v>74</v>
       </c>
       <c r="E71" s="2"/>
       <c r="F71" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G71" t="s" s="2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H71" t="s" s="2">
         <v>74</v>
       </c>
       <c r="I71" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J71" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K71" t="s" s="2">
-        <v>104</v>
+        <v>395</v>
       </c>
       <c r="L71" t="s" s="2">
-        <v>229</v>
+        <v>396</v>
       </c>
       <c r="M71" t="s" s="2">
-        <v>230</v>
+        <v>397</v>
       </c>
       <c r="N71" t="s" s="2">
-        <v>107</v>
+        <v>216</v>
       </c>
       <c r="O71" t="s" s="2">
-        <v>202</v>
+        <v>398</v>
       </c>
       <c r="P71" t="s" s="2">
         <v>74</v>
@@ -9755,25 +9588,25 @@
         <v>74</v>
       </c>
       <c r="AF71" t="s" s="2">
-        <v>231</v>
+        <v>394</v>
       </c>
       <c r="AG71" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH71" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI71" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ71" t="s" s="2">
-        <v>112</v>
+        <v>217</v>
       </c>
       <c r="AK71" t="s" s="2">
-        <v>95</v>
+        <v>399</v>
       </c>
       <c r="AL71" t="s" s="2">
-        <v>74</v>
+        <v>400</v>
       </c>
       <c r="AM71" t="s" s="2">
         <v>74</v>
@@ -9781,14 +9614,14 @@
     </row>
     <row r="72">
       <c r="A72" t="s" s="2">
-        <v>417</v>
+        <v>401</v>
       </c>
       <c r="B72" t="s" s="2">
-        <v>417</v>
+        <v>401</v>
       </c>
       <c r="C72" s="2"/>
       <c r="D72" t="s" s="2">
-        <v>326</v>
+        <v>74</v>
       </c>
       <c r="E72" s="2"/>
       <c r="F72" t="s" s="2">
@@ -9807,16 +9640,16 @@
         <v>74</v>
       </c>
       <c r="K72" t="s" s="2">
-        <v>282</v>
+        <v>402</v>
       </c>
       <c r="L72" t="s" s="2">
-        <v>418</v>
+        <v>403</v>
       </c>
       <c r="M72" t="s" s="2">
-        <v>419</v>
+        <v>404</v>
       </c>
       <c r="N72" t="s" s="2">
-        <v>285</v>
+        <v>405</v>
       </c>
       <c r="O72" s="2"/>
       <c r="P72" t="s" s="2">
@@ -9866,7 +9699,7 @@
         <v>74</v>
       </c>
       <c r="AF72" t="s" s="2">
-        <v>417</v>
+        <v>401</v>
       </c>
       <c r="AG72" t="s" s="2">
         <v>75</v>
@@ -9878,13 +9711,13 @@
         <v>93</v>
       </c>
       <c r="AJ72" t="s" s="2">
-        <v>94</v>
+        <v>217</v>
       </c>
       <c r="AK72" t="s" s="2">
-        <v>288</v>
+        <v>406</v>
       </c>
       <c r="AL72" t="s" s="2">
-        <v>74</v>
+        <v>407</v>
       </c>
       <c r="AM72" t="s" s="2">
         <v>74</v>
@@ -9892,10 +9725,10 @@
     </row>
     <row r="73">
       <c r="A73" t="s" s="2">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="B73" t="s" s="2">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="C73" s="2"/>
       <c r="D73" t="s" s="2">
@@ -9906,7 +9739,7 @@
         <v>75</v>
       </c>
       <c r="G73" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H73" t="s" s="2">
         <v>74</v>
@@ -9918,15 +9751,17 @@
         <v>74</v>
       </c>
       <c r="K73" t="s" s="2">
-        <v>205</v>
+        <v>409</v>
       </c>
       <c r="L73" t="s" s="2">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="M73" t="s" s="2">
-        <v>422</v>
-      </c>
-      <c r="N73" s="2"/>
+        <v>411</v>
+      </c>
+      <c r="N73" t="s" s="2">
+        <v>412</v>
+      </c>
       <c r="O73" s="2"/>
       <c r="P73" t="s" s="2">
         <v>74</v>
@@ -9975,25 +9810,25 @@
         <v>74</v>
       </c>
       <c r="AF73" t="s" s="2">
-        <v>420</v>
+        <v>408</v>
       </c>
       <c r="AG73" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH73" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI73" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ73" t="s" s="2">
-        <v>94</v>
+        <v>413</v>
       </c>
       <c r="AK73" t="s" s="2">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="AL73" t="s" s="2">
-        <v>238</v>
+        <v>407</v>
       </c>
       <c r="AM73" t="s" s="2">
         <v>74</v>
@@ -10001,10 +9836,10 @@
     </row>
     <row r="74">
       <c r="A74" t="s" s="2">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="B74" t="s" s="2">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="C74" s="2"/>
       <c r="D74" t="s" s="2">
@@ -10012,10 +9847,10 @@
       </c>
       <c r="E74" s="2"/>
       <c r="F74" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="G74" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H74" t="s" s="2">
         <v>74</v>
@@ -10027,18 +9862,20 @@
         <v>74</v>
       </c>
       <c r="K74" t="s" s="2">
-        <v>97</v>
+        <v>416</v>
       </c>
       <c r="L74" t="s" s="2">
-        <v>425</v>
+        <v>417</v>
       </c>
       <c r="M74" t="s" s="2">
-        <v>426</v>
+        <v>418</v>
       </c>
       <c r="N74" t="s" s="2">
-        <v>236</v>
-      </c>
-      <c r="O74" s="2"/>
+        <v>216</v>
+      </c>
+      <c r="O74" t="s" s="2">
+        <v>419</v>
+      </c>
       <c r="P74" t="s" s="2">
         <v>74</v>
       </c>
@@ -10086,10 +9923,10 @@
         <v>74</v>
       </c>
       <c r="AF74" t="s" s="2">
-        <v>424</v>
+        <v>415</v>
       </c>
       <c r="AG74" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="AH74" t="s" s="2">
         <v>81</v>
@@ -10098,13 +9935,13 @@
         <v>93</v>
       </c>
       <c r="AJ74" t="s" s="2">
-        <v>94</v>
+        <v>217</v>
       </c>
       <c r="AK74" t="s" s="2">
-        <v>101</v>
+        <v>420</v>
       </c>
       <c r="AL74" t="s" s="2">
-        <v>74</v>
+        <v>421</v>
       </c>
       <c r="AM74" t="s" s="2">
         <v>74</v>
@@ -10112,10 +9949,10 @@
     </row>
     <row r="75">
       <c r="A75" t="s" s="2">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="B75" t="s" s="2">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" t="s" s="2">
@@ -10138,15 +9975,17 @@
         <v>74</v>
       </c>
       <c r="K75" t="s" s="2">
-        <v>220</v>
+        <v>125</v>
       </c>
       <c r="L75" t="s" s="2">
-        <v>428</v>
+        <v>423</v>
       </c>
       <c r="M75" t="s" s="2">
-        <v>429</v>
-      </c>
-      <c r="N75" s="2"/>
+        <v>424</v>
+      </c>
+      <c r="N75" t="s" s="2">
+        <v>425</v>
+      </c>
       <c r="O75" s="2"/>
       <c r="P75" t="s" s="2">
         <v>74</v>
@@ -10195,13 +10034,13 @@
         <v>74</v>
       </c>
       <c r="AF75" t="s" s="2">
-        <v>427</v>
+        <v>422</v>
       </c>
       <c r="AG75" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH75" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI75" t="s" s="2">
         <v>93</v>
@@ -10210,10 +10049,10 @@
         <v>94</v>
       </c>
       <c r="AK75" t="s" s="2">
-        <v>101</v>
+        <v>426</v>
       </c>
       <c r="AL75" t="s" s="2">
-        <v>74</v>
+        <v>421</v>
       </c>
       <c r="AM75" t="s" s="2">
         <v>74</v>
@@ -10221,10 +10060,10 @@
     </row>
     <row r="76">
       <c r="A76" t="s" s="2">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="B76" t="s" s="2">
-        <v>430</v>
+        <v>427</v>
       </c>
       <c r="C76" s="2"/>
       <c r="D76" t="s" s="2">
@@ -10235,7 +10074,7 @@
         <v>75</v>
       </c>
       <c r="G76" t="s" s="2">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="H76" t="s" s="2">
         <v>74</v>
@@ -10247,15 +10086,17 @@
         <v>74</v>
       </c>
       <c r="K76" t="s" s="2">
-        <v>97</v>
+        <v>428</v>
       </c>
       <c r="L76" t="s" s="2">
-        <v>98</v>
+        <v>429</v>
       </c>
       <c r="M76" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N76" s="2"/>
+        <v>430</v>
+      </c>
+      <c r="N76" t="s" s="2">
+        <v>431</v>
+      </c>
       <c r="O76" s="2"/>
       <c r="P76" t="s" s="2">
         <v>74</v>
@@ -10304,22 +10145,22 @@
         <v>74</v>
       </c>
       <c r="AF76" t="s" s="2">
-        <v>100</v>
+        <v>427</v>
       </c>
       <c r="AG76" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH76" t="s" s="2">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="AI76" t="s" s="2">
-        <v>74</v>
+        <v>93</v>
       </c>
       <c r="AJ76" t="s" s="2">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="AK76" t="s" s="2">
-        <v>101</v>
+        <v>432</v>
       </c>
       <c r="AL76" t="s" s="2">
         <v>74</v>
@@ -10330,21 +10171,21 @@
     </row>
     <row r="77">
       <c r="A77" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B77" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C77" s="2"/>
       <c r="D77" t="s" s="2">
-        <v>103</v>
+        <v>74</v>
       </c>
       <c r="E77" s="2"/>
       <c r="F77" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G77" t="s" s="2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H77" t="s" s="2">
         <v>74</v>
@@ -10353,19 +10194,19 @@
         <v>74</v>
       </c>
       <c r="J77" t="s" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="K77" t="s" s="2">
-        <v>104</v>
+        <v>282</v>
       </c>
       <c r="L77" t="s" s="2">
-        <v>105</v>
+        <v>434</v>
       </c>
       <c r="M77" t="s" s="2">
-        <v>106</v>
+        <v>435</v>
       </c>
       <c r="N77" t="s" s="2">
-        <v>107</v>
+        <v>285</v>
       </c>
       <c r="O77" s="2"/>
       <c r="P77" t="s" s="2">
@@ -10403,19 +10244,19 @@
         <v>74</v>
       </c>
       <c r="AB77" t="s" s="2">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="AC77" t="s" s="2">
-        <v>109</v>
+        <v>74</v>
       </c>
       <c r="AD77" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AE77" t="s" s="2">
-        <v>110</v>
+        <v>74</v>
       </c>
       <c r="AF77" t="s" s="2">
-        <v>111</v>
+        <v>433</v>
       </c>
       <c r="AG77" t="s" s="2">
         <v>75</v>
@@ -10427,10 +10268,10 @@
         <v>93</v>
       </c>
       <c r="AJ77" t="s" s="2">
-        <v>112</v>
+        <v>94</v>
       </c>
       <c r="AK77" t="s" s="2">
-        <v>95</v>
+        <v>272</v>
       </c>
       <c r="AL77" t="s" s="2">
         <v>74</v>
@@ -10441,46 +10282,44 @@
     </row>
     <row r="78">
       <c r="A78" t="s" s="2">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="B78" t="s" s="2">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="C78" s="2"/>
       <c r="D78" t="s" s="2">
-        <v>228</v>
+        <v>74</v>
       </c>
       <c r="E78" s="2"/>
       <c r="F78" t="s" s="2">
         <v>75</v>
       </c>
       <c r="G78" t="s" s="2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H78" t="s" s="2">
         <v>74</v>
       </c>
       <c r="I78" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="J78" t="s" s="2">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="K78" t="s" s="2">
-        <v>104</v>
+        <v>437</v>
       </c>
       <c r="L78" t="s" s="2">
-        <v>229</v>
+        <v>438</v>
       </c>
       <c r="M78" t="s" s="2">
-        <v>230</v>
+        <v>439</v>
       </c>
       <c r="N78" t="s" s="2">
-        <v>107</v>
-      </c>
-      <c r="O78" t="s" s="2">
-        <v>202</v>
-      </c>
+        <v>216</v>
+      </c>
+      <c r="O78" s="2"/>
       <c r="P78" t="s" s="2">
         <v>74</v>
       </c>
@@ -10528,1252 +10367,27 @@
         <v>74</v>
       </c>
       <c r="AF78" t="s" s="2">
-        <v>231</v>
+        <v>436</v>
       </c>
       <c r="AG78" t="s" s="2">
         <v>75</v>
       </c>
       <c r="AH78" t="s" s="2">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="AI78" t="s" s="2">
         <v>93</v>
       </c>
       <c r="AJ78" t="s" s="2">
-        <v>112</v>
+        <v>217</v>
       </c>
       <c r="AK78" t="s" s="2">
-        <v>95</v>
+        <v>218</v>
       </c>
       <c r="AL78" t="s" s="2">
         <v>74</v>
       </c>
       <c r="AM78" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="B79" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="C79" s="2"/>
-      <c r="D79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E79" s="2"/>
-      <c r="F79" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="G79" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K79" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="L79" t="s" s="2">
-        <v>434</v>
-      </c>
-      <c r="M79" t="s" s="2">
-        <v>435</v>
-      </c>
-      <c r="N79" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="O79" s="2"/>
-      <c r="P79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q79" s="2"/>
-      <c r="R79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF79" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="AG79" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AH79" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI79" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ79" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AK79" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="AL79" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM79" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="s" s="2">
-        <v>436</v>
-      </c>
-      <c r="B80" t="s" s="2">
-        <v>436</v>
-      </c>
-      <c r="C80" s="2"/>
-      <c r="D80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E80" s="2"/>
-      <c r="F80" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G80" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K80" t="s" s="2">
-        <v>437</v>
-      </c>
-      <c r="L80" t="s" s="2">
-        <v>438</v>
-      </c>
-      <c r="M80" t="s" s="2">
-        <v>439</v>
-      </c>
-      <c r="N80" t="s" s="2">
-        <v>440</v>
-      </c>
-      <c r="O80" s="2"/>
-      <c r="P80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q80" s="2"/>
-      <c r="R80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF80" t="s" s="2">
-        <v>436</v>
-      </c>
-      <c r="AG80" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH80" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI80" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ80" t="s" s="2">
-        <v>441</v>
-      </c>
-      <c r="AK80" t="s" s="2">
-        <v>442</v>
-      </c>
-      <c r="AL80" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM80" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="s" s="2">
-        <v>443</v>
-      </c>
-      <c r="B81" t="s" s="2">
-        <v>443</v>
-      </c>
-      <c r="C81" s="2"/>
-      <c r="D81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E81" s="2"/>
-      <c r="F81" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G81" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="H81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K81" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="L81" t="s" s="2">
-        <v>444</v>
-      </c>
-      <c r="M81" t="s" s="2">
-        <v>445</v>
-      </c>
-      <c r="N81" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="O81" s="2"/>
-      <c r="P81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q81" s="2"/>
-      <c r="R81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF81" t="s" s="2">
-        <v>443</v>
-      </c>
-      <c r="AG81" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH81" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI81" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ81" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AK81" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="AL81" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM81" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="s" s="2">
-        <v>446</v>
-      </c>
-      <c r="B82" t="s" s="2">
-        <v>446</v>
-      </c>
-      <c r="C82" s="2"/>
-      <c r="D82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E82" s="2"/>
-      <c r="F82" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G82" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K82" t="s" s="2">
-        <v>447</v>
-      </c>
-      <c r="L82" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="M82" t="s" s="2">
-        <v>449</v>
-      </c>
-      <c r="N82" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="O82" t="s" s="2">
-        <v>450</v>
-      </c>
-      <c r="P82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q82" s="2"/>
-      <c r="R82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE82" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF82" t="s" s="2">
-        <v>446</v>
-      </c>
-      <c r="AG82" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH82" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI82" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ82" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="AK82" t="s" s="2">
-        <v>451</v>
-      </c>
-      <c r="AL82" t="s" s="2">
-        <v>452</v>
-      </c>
-      <c r="AM82" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="B83" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="C83" s="2"/>
-      <c r="D83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E83" s="2"/>
-      <c r="F83" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G83" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="H83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K83" t="s" s="2">
-        <v>454</v>
-      </c>
-      <c r="L83" t="s" s="2">
-        <v>455</v>
-      </c>
-      <c r="M83" t="s" s="2">
-        <v>456</v>
-      </c>
-      <c r="N83" t="s" s="2">
-        <v>457</v>
-      </c>
-      <c r="O83" s="2"/>
-      <c r="P83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q83" s="2"/>
-      <c r="R83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE83" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF83" t="s" s="2">
-        <v>453</v>
-      </c>
-      <c r="AG83" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH83" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI83" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ83" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="AK83" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="AL83" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="AM83" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="B84" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="C84" s="2"/>
-      <c r="D84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E84" s="2"/>
-      <c r="F84" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G84" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K84" t="s" s="2">
-        <v>461</v>
-      </c>
-      <c r="L84" t="s" s="2">
-        <v>462</v>
-      </c>
-      <c r="M84" t="s" s="2">
-        <v>463</v>
-      </c>
-      <c r="N84" t="s" s="2">
-        <v>464</v>
-      </c>
-      <c r="O84" s="2"/>
-      <c r="P84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q84" s="2"/>
-      <c r="R84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE84" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF84" t="s" s="2">
-        <v>460</v>
-      </c>
-      <c r="AG84" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH84" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI84" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ84" t="s" s="2">
-        <v>465</v>
-      </c>
-      <c r="AK84" t="s" s="2">
-        <v>466</v>
-      </c>
-      <c r="AL84" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="AM84" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="B85" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="C85" s="2"/>
-      <c r="D85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E85" s="2"/>
-      <c r="F85" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G85" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K85" t="s" s="2">
-        <v>468</v>
-      </c>
-      <c r="L85" t="s" s="2">
-        <v>469</v>
-      </c>
-      <c r="M85" t="s" s="2">
-        <v>470</v>
-      </c>
-      <c r="N85" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="O85" t="s" s="2">
-        <v>471</v>
-      </c>
-      <c r="P85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q85" s="2"/>
-      <c r="R85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE85" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF85" t="s" s="2">
-        <v>467</v>
-      </c>
-      <c r="AG85" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH85" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI85" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ85" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="AK85" t="s" s="2">
-        <v>472</v>
-      </c>
-      <c r="AL85" t="s" s="2">
-        <v>473</v>
-      </c>
-      <c r="AM85" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="s" s="2">
-        <v>474</v>
-      </c>
-      <c r="B86" t="s" s="2">
-        <v>474</v>
-      </c>
-      <c r="C86" s="2"/>
-      <c r="D86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E86" s="2"/>
-      <c r="F86" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G86" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K86" t="s" s="2">
-        <v>125</v>
-      </c>
-      <c r="L86" t="s" s="2">
-        <v>475</v>
-      </c>
-      <c r="M86" t="s" s="2">
-        <v>476</v>
-      </c>
-      <c r="N86" t="s" s="2">
-        <v>477</v>
-      </c>
-      <c r="O86" s="2"/>
-      <c r="P86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q86" s="2"/>
-      <c r="R86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE86" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF86" t="s" s="2">
-        <v>474</v>
-      </c>
-      <c r="AG86" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH86" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI86" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ86" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AK86" t="s" s="2">
-        <v>478</v>
-      </c>
-      <c r="AL86" t="s" s="2">
-        <v>473</v>
-      </c>
-      <c r="AM86" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="s" s="2">
-        <v>479</v>
-      </c>
-      <c r="B87" t="s" s="2">
-        <v>479</v>
-      </c>
-      <c r="C87" s="2"/>
-      <c r="D87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E87" s="2"/>
-      <c r="F87" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G87" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K87" t="s" s="2">
-        <v>480</v>
-      </c>
-      <c r="L87" t="s" s="2">
-        <v>481</v>
-      </c>
-      <c r="M87" t="s" s="2">
-        <v>482</v>
-      </c>
-      <c r="N87" t="s" s="2">
-        <v>483</v>
-      </c>
-      <c r="O87" s="2"/>
-      <c r="P87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q87" s="2"/>
-      <c r="R87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF87" t="s" s="2">
-        <v>479</v>
-      </c>
-      <c r="AG87" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH87" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI87" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ87" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AK87" t="s" s="2">
-        <v>484</v>
-      </c>
-      <c r="AL87" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM87" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="B88" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="C88" s="2"/>
-      <c r="D88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E88" s="2"/>
-      <c r="F88" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G88" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J88" t="s" s="2">
-        <v>82</v>
-      </c>
-      <c r="K88" t="s" s="2">
-        <v>282</v>
-      </c>
-      <c r="L88" t="s" s="2">
-        <v>486</v>
-      </c>
-      <c r="M88" t="s" s="2">
-        <v>487</v>
-      </c>
-      <c r="N88" t="s" s="2">
-        <v>285</v>
-      </c>
-      <c r="O88" s="2"/>
-      <c r="P88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q88" s="2"/>
-      <c r="R88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF88" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="AG88" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH88" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AI88" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ88" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="AK88" t="s" s="2">
-        <v>272</v>
-      </c>
-      <c r="AL88" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM88" t="s" s="2">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="B89" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="C89" s="2"/>
-      <c r="D89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="E89" s="2"/>
-      <c r="F89" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="G89" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="H89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="I89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="J89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="K89" t="s" s="2">
-        <v>489</v>
-      </c>
-      <c r="L89" t="s" s="2">
-        <v>490</v>
-      </c>
-      <c r="M89" t="s" s="2">
-        <v>491</v>
-      </c>
-      <c r="N89" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="O89" s="2"/>
-      <c r="P89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Q89" s="2"/>
-      <c r="R89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="S89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="T89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="U89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="V89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="W89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="X89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Y89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="Z89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AA89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AB89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AC89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AD89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AE89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AF89" t="s" s="2">
-        <v>488</v>
-      </c>
-      <c r="AG89" t="s" s="2">
-        <v>75</v>
-      </c>
-      <c r="AH89" t="s" s="2">
-        <v>81</v>
-      </c>
-      <c r="AI89" t="s" s="2">
-        <v>93</v>
-      </c>
-      <c r="AJ89" t="s" s="2">
-        <v>217</v>
-      </c>
-      <c r="AK89" t="s" s="2">
-        <v>218</v>
-      </c>
-      <c r="AL89" t="s" s="2">
-        <v>74</v>
-      </c>
-      <c r="AM89" t="s" s="2">
         <v>74</v>
       </c>
     </row>

</xml_diff>